<commit_message>
Actualizacion de Logger y plantilla
</commit_message>
<xml_diff>
--- a/data/empresas.xlsx
+++ b/data/empresas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/andres_ramirez_virtualsoft_tech/Documents/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andres Ramirez\Documents\2026\automatizacionGmaill\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4338CBC-561C-4EF0-AF44-3457DD0A96EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2533BE-7364-41AC-9FDB-ECB31909552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{2713CE67-7A45-453D-B01E-A4D3FC556313}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2713CE67-7A45-453D-B01E-A4D3FC556313}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Empresa</t>
   </si>
@@ -47,22 +47,184 @@
     <t>Correo</t>
   </si>
   <si>
-    <t>LeoVegas</t>
-  </si>
-  <si>
-    <t>correo1@empresa.com</t>
-  </si>
-  <si>
-    <t>EveryMatrix</t>
-  </si>
-  <si>
-    <t>correo2@empresa.com</t>
-  </si>
-  <si>
-    <t>Betsson</t>
-  </si>
-  <si>
-    <t>correo3@empresa.com</t>
+    <t>Sixtema</t>
+  </si>
+  <si>
+    <t>rrhh@sixtema.es</t>
+  </si>
+  <si>
+    <t>CustomerTop</t>
+  </si>
+  <si>
+    <t>rrhh@customertop.es</t>
+  </si>
+  <si>
+    <t>AVC Tech Solutions</t>
+  </si>
+  <si>
+    <t>rrhh@avctechsolutions.com</t>
+  </si>
+  <si>
+    <t>BOTECH</t>
+  </si>
+  <si>
+    <t>rrhh@botech.info</t>
+  </si>
+  <si>
+    <t>Experian CheetahMail</t>
+  </si>
+  <si>
+    <t>rrhh@experian-cheetahmail.es</t>
+  </si>
+  <si>
+    <t>Abemon</t>
+  </si>
+  <si>
+    <t>rrhh@abemon.es</t>
+  </si>
+  <si>
+    <t>Bequant</t>
+  </si>
+  <si>
+    <t>jobs@bequant.com</t>
+  </si>
+  <si>
+    <t>Esri España</t>
+  </si>
+  <si>
+    <t>rrhh@esri.es</t>
+  </si>
+  <si>
+    <t>Voz.com</t>
+  </si>
+  <si>
+    <t>rrhh@voz.com</t>
+  </si>
+  <si>
+    <t>GlobalTel</t>
+  </si>
+  <si>
+    <t>rrhh@globaltel.es</t>
+  </si>
+  <si>
+    <t>Dayvo</t>
+  </si>
+  <si>
+    <t>rrhh@dayvo.com</t>
+  </si>
+  <si>
+    <t>Geotelecom</t>
+  </si>
+  <si>
+    <t>rrhh@geotelecom.es</t>
+  </si>
+  <si>
+    <t>HPS</t>
+  </si>
+  <si>
+    <t>rrhh@hps.es</t>
+  </si>
+  <si>
+    <t>STI Soluciones Tecnológicas</t>
+  </si>
+  <si>
+    <t>rrhh@sti-sl.es</t>
+  </si>
+  <si>
+    <t>Adtel</t>
+  </si>
+  <si>
+    <t>rrhh@adtel.es</t>
+  </si>
+  <si>
+    <t>Signe</t>
+  </si>
+  <si>
+    <t>rrhh@signe.es</t>
+  </si>
+  <si>
+    <t>VASS</t>
+  </si>
+  <si>
+    <t>rrhh@vass.es</t>
+  </si>
+  <si>
+    <t>GMV</t>
+  </si>
+  <si>
+    <t>careers@gmv.com</t>
+  </si>
+  <si>
+    <t>Plain Concepts</t>
+  </si>
+  <si>
+    <t>jobs@plainconcepts.com</t>
+  </si>
+  <si>
+    <t>Babel</t>
+  </si>
+  <si>
+    <t>careers@babelgroup.com</t>
+  </si>
+  <si>
+    <t>Netmind</t>
+  </si>
+  <si>
+    <t>jobs@netmind.net</t>
+  </si>
+  <si>
+    <t>Cognodata</t>
+  </si>
+  <si>
+    <t>jobs@cognodata.com</t>
+  </si>
+  <si>
+    <t>Izertis</t>
+  </si>
+  <si>
+    <t>empleo@izertis.com</t>
+  </si>
+  <si>
+    <t>Sngular</t>
+  </si>
+  <si>
+    <t>careers@sngular.com</t>
+  </si>
+  <si>
+    <t>knowmad mood</t>
+  </si>
+  <si>
+    <t>jobs@knowmadmood.com</t>
+  </si>
+  <si>
+    <t>OPPLUS</t>
+  </si>
+  <si>
+    <t>talent@opplus.es</t>
+  </si>
+  <si>
+    <t>BySidecar</t>
+  </si>
+  <si>
+    <t>careers@bysidecar.com</t>
+  </si>
+  <si>
+    <t>Factorial</t>
+  </si>
+  <si>
+    <t>info@factorial.co</t>
+  </si>
+  <si>
+    <t>CIEM Systems</t>
+  </si>
+  <si>
+    <t>info@ciemsystems.eu</t>
+  </si>
+  <si>
+    <t>Mentor VR</t>
+  </si>
+  <si>
+    <t>hola@mentor-vr.com</t>
   </si>
 </sst>
 </file>
@@ -461,8 +623,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538A5E57-67B4-4B95-851D-923762D11352}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="47.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -472,7 +637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -480,7 +645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -496,11 +661,254 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="mailto:correo1@empresa.com" xr:uid="{7FE7D221-6E0B-405F-AF88-0A1F8BBA0339}"/>
-    <hyperlink ref="B3" r:id="rId2" display="mailto:correo2@empresa.com" xr:uid="{10F59890-B1A4-433A-9E86-12A256EA43D5}"/>
-    <hyperlink ref="B4" r:id="rId3" display="mailto:correo3@empresa.com" xr:uid="{B5FC1DEB-223B-4957-8F9B-4BA186B3A48F}"/>
+    <hyperlink ref="B2" r:id="rId1" display="mailto:rrhh@sixtema.es" xr:uid="{54E8297C-D6EF-4016-9DB8-3A0B38EA6F06}"/>
+    <hyperlink ref="B3" r:id="rId2" display="mailto:rrhh@customertop.es" xr:uid="{A5685496-9C33-495C-BA57-82930C7FCA18}"/>
+    <hyperlink ref="B4" r:id="rId3" display="mailto:rrhh@avctechsolutions.com" xr:uid="{AB7668C5-6186-4328-9C5F-75172AB4CA7D}"/>
+    <hyperlink ref="B5" r:id="rId4" display="mailto:rrhh@botech.info" xr:uid="{E7A14F75-81FF-4299-A346-7AB552F6E1E4}"/>
+    <hyperlink ref="B6" r:id="rId5" display="mailto:rrhh@experian-cheetahmail.es" xr:uid="{50671CC5-EB3A-4651-A063-4013A7AA4106}"/>
+    <hyperlink ref="B7" r:id="rId6" display="mailto:rrhh@abemon.es" xr:uid="{88DEC044-E22B-415D-8925-25FA9B6B3F89}"/>
+    <hyperlink ref="B8" r:id="rId7" display="mailto:jobs@bequant.com" xr:uid="{7F40A34C-C0B2-4B9C-AAB8-3E7C687DCDEF}"/>
+    <hyperlink ref="B9" r:id="rId8" display="mailto:rrhh@esri.es" xr:uid="{B03B4345-A073-4EF9-8782-D77C0E5B35BD}"/>
+    <hyperlink ref="B10" r:id="rId9" display="mailto:rrhh@voz.com" xr:uid="{ED9B837D-3CBE-48D7-9E8C-38E6B4155BE8}"/>
+    <hyperlink ref="B11" r:id="rId10" display="mailto:rrhh@globaltel.es" xr:uid="{216C71A8-956E-4C0C-8A95-D0C72CDA26CE}"/>
+    <hyperlink ref="B12" r:id="rId11" display="mailto:rrhh@dayvo.com" xr:uid="{E3D5C827-1386-4001-BE71-413D89D15613}"/>
+    <hyperlink ref="B13" r:id="rId12" display="mailto:rrhh@geotelecom.es" xr:uid="{19EBF594-C7AC-4C92-85DA-26A183539119}"/>
+    <hyperlink ref="B14" r:id="rId13" display="mailto:rrhh@hps.es" xr:uid="{A63F91EF-011D-407F-83CB-D9E53952EFED}"/>
+    <hyperlink ref="B15" r:id="rId14" display="mailto:rrhh@sti-sl.es" xr:uid="{8C5E9749-D946-41FD-840B-21E969FC3C98}"/>
+    <hyperlink ref="B16" r:id="rId15" display="mailto:rrhh@adtel.es" xr:uid="{B1388B0A-37DC-47B8-A756-D4495EDF7080}"/>
+    <hyperlink ref="B17" r:id="rId16" display="mailto:rrhh@signe.es" xr:uid="{C4EF56FF-4722-4266-8EAA-EA6B3A0A7BD3}"/>
+    <hyperlink ref="B18" r:id="rId17" display="mailto:rrhh@vass.es" xr:uid="{D963AE44-8326-4079-A6A5-D7983CE8811C}"/>
+    <hyperlink ref="B19" r:id="rId18" display="mailto:careers@gmv.com" xr:uid="{D4A25C5D-CF19-404E-BC7D-48AE2506E1F2}"/>
+    <hyperlink ref="B20" r:id="rId19" display="mailto:jobs@plainconcepts.com" xr:uid="{DF18DF72-D1DA-4B04-B9E7-67E0C617A9D9}"/>
+    <hyperlink ref="B21" r:id="rId20" display="mailto:careers@babelgroup.com" xr:uid="{6CF55E7C-F947-4263-9BEA-CDD0B77BE194}"/>
+    <hyperlink ref="B22" r:id="rId21" display="mailto:jobs@netmind.net" xr:uid="{2FE6AB0D-C0A7-4C4D-B81D-B619DE158C67}"/>
+    <hyperlink ref="B23" r:id="rId22" display="mailto:jobs@cognodata.com" xr:uid="{9183010A-C839-4F3A-8CDB-F500CCF07A2F}"/>
+    <hyperlink ref="B24" r:id="rId23" display="mailto:empleo@izertis.com" xr:uid="{F194E098-6A21-4870-BA1C-DF9B4418FDA3}"/>
+    <hyperlink ref="B25" r:id="rId24" display="mailto:careers@sngular.com" xr:uid="{3800EEC8-8813-4ACA-8BEA-3E7EAFF542C0}"/>
+    <hyperlink ref="B26" r:id="rId25" display="mailto:jobs@knowmadmood.com" xr:uid="{259A173D-F9EF-4552-99CE-28E6AEE33A84}"/>
+    <hyperlink ref="B27" r:id="rId26" display="mailto:talent@opplus.es" xr:uid="{CC410333-7F06-4BD2-AC6C-D21C3E2CB79D}"/>
+    <hyperlink ref="B28" r:id="rId27" display="mailto:careers@bysidecar.com" xr:uid="{4A082D17-178B-44A2-9A2A-2EE85471EE5F}"/>
+    <hyperlink ref="B29" r:id="rId28" display="mailto:info@factorial.co" xr:uid="{E3E6FBBA-D929-4460-BA84-1451A60A8236}"/>
+    <hyperlink ref="B30" r:id="rId29" display="mailto:info@ciemsystems.eu" xr:uid="{9A90C928-FB88-4046-B335-57E2D89953C7}"/>
+    <hyperlink ref="B31" r:id="rId30" display="mailto:hola@mentor-vr.com" xr:uid="{FDFE9400-BF01-4343-9788-C73D8E2B0742}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>